<commit_message>
enemy phase end crash
crashing at the end of enemy phase, after all enemies have moved but before enemy phase actually ends
</commit_message>
<xml_diff>
--- a/chapter_items.xlsx
+++ b/chapter_items.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -553,7 +553,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ch3Armory: IronBlade, SteelSword, SteelLance, SteelAxe, SlimLance, SlimAxe, Javelin, HandAxe, Hammer | Ch3Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
+          <t>Ch5Armory: IronBlade, SteelSword, SteelLance, SteelAxe, SlimLance, SlimAxe, Javelin, HandAxe, Hammer | Ch5Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
         </is>
       </c>
     </row>
@@ -583,14 +583,14 @@
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ChapterEventsInstaller</t>
+          <t>Ch7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -598,12 +598,16 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ch7Armory: IronBlade, SteelSword, SteelLance, SteelAxe, SlimLance, SlimAxe, Javelin, HandAxe, Hammer | Ch7Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Epilogue</t>
+          <t>ChapterEventsInstaller</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -616,7 +620,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GenericEvents</t>
+          <t>Epilogue</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -625,6 +629,19 @@
         <v>0</v>
       </c>
       <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GenericEvents</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
ch 7 akashic bow, portraits
</commit_message>
<xml_diff>
--- a/chapter_items.xlsx
+++ b/chapter_items.xlsx
@@ -593,14 +593,18 @@
           <t>Ch7</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AkashicBow, KillerBow</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ch7Armory: IronBlade, SteelSword, SteelLance, SteelAxe, SlimLance, SlimAxe, Javelin, HandAxe, Hammer | Ch7Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
+          <t>Ch7Armory: IronBlade, SteelSword, SteelLance, SteelAxe, SlimLance, SlimAxe, KillerBow, KillingEdge, Javelin, HandAxe, Hammer | Ch7Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ch 7 akashic bow, portraits, guide
</commit_message>
<xml_diff>
--- a/chapter_items.xlsx
+++ b/chapter_items.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AblatioPhoton x2, Angel x2, Breeze x2, Elfire x2, Key, PatientKatti x2, Quickblade x2, Rescue x2, Restore, SilverSword, SteelSword x2</t>
+          <t>AblatioPhoton x2, Angel x2, Breeze x2, Elfire x2, Heal x2, IronSword x2, Key, PatientKatti x2, Quickblade x2, Rescue x2, Restore, SilverSword, SteelSword x2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -566,7 +566,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ch7Armory: IronBlade, SteelSword, SteelLance, SteelAxe, SlimLance, SlimAxe, KillerBow, KillingEdge, Javelin, HandAxe, Hammer | Ch7Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
+          <t>Ch7Armory: SteelBlade, SteelSword, SteelLance, SteelAxe, SlimLance, KillerAxe, KillerBow, KillingEdge, Javelin, HandAxe, Hammer | Ch7Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ch 6 and 7 dev
</commit_message>
<xml_diff>
--- a/chapter_items.xlsx
+++ b/chapter_items.xlsx
@@ -581,9 +581,13 @@
           <t>CyclonicLance, Fire x2, IronLance x2, SteelBlade x2, Thunder x2, Vulnerary x2</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Butterfly OR Lancereaver</t>
+        </is>
+      </c>
       <c r="D8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
@@ -595,7 +599,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AkashicBow, Loneliness</t>
+          <t>AkashicBow, Butterfly, Loneliness</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -604,7 +608,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ch7Armory: SteelBlade, SteelSword, SteelLance, SteelAxe, SlimLance, KillerAxe, KillerBow, KillingEdge, Javelin, HandAxe, Hammer | Ch7Vendor: Fire, Thunder, Pain, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
+          <t>Ch7Armory: SteelBlade, SteelSword, SteelLance, SteelAxe, SlimLance, KillerAxe, KillerLance, KillingEdge, Swordreaver, Javelin, HandAxe, Hammer | Ch7Vendor: Fire, Thunder, Light, Pain, Exploitation, Heal, Mend, Restore, Torch, HeavyBomb, RedHornet</t>
         </is>
       </c>
     </row>

</xml_diff>